<commit_message>
Adding results and analysis scripts to generate plots
</commit_message>
<xml_diff>
--- a/questionnaire/questionnaire-data.xlsx
+++ b/questionnaire/questionnaire-data.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="263">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -712,6 +712,142 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">I would add the number of lines into the radar</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">5 to 10 years</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#4 Optimize parameter matching in TableMetaDataContext;#10 35626: defaultCandidate for scoped proxies;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#12 Refactor doGetBeanNamesForType for improved readability and performance;#6 Add QUERY HTTP method;#7 Add RSocketServiceMethod support for Kotlin suspending functions;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#7 Add RSocketServiceMethod support for Kotlin suspending functions </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pouvoir se faire une idée de la complexité d'une MR avant de choisir laquelle revoir</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">parfois le plugin se trompe, pas forcément facile de trouver les bons critères sans se retrouver avec 15 critères</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">nombre de fichiers (en retirant code "simple"/commentaire)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Files count;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">essayer d'autres métrique/adapter les métrique</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Chouette idée!</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#10 35626: defaultCandidate for scoped proxies;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#4 Optimize parameter matching in TableMetaDataContext;#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#7 Add RSocketServiceMethod support for Kotlin suspending functions;#12 Refactor doGetBeanNamesForType for improved readability and performance;#6 Add QUERY HTTP method;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Confident</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Je ne comprends pas quels critères ont été utilisés pour classer cette PR #4 aussi loin alors qu'elle est bien documentée, qu'il y a peu de fichiers et lignes de code modifiés. Bien qu'il n'y ait pas de tests, cette PR semble pouvoir être résolue plus rapidement.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#6 Add QUERY HTTP method</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Combining several metrics in a single visualization</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Time to compute the visualization making the switching between PR difficult. It would help to make it faster in to encourage the comparison. </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Context switching between files. Any other would be welcomed, especially if it's customizable.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Same comment that 51.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">I would like to have an overall (holistic) visualization gathering or presenting all the radar charts at a glance.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Push for it, that's great!</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3 to 5 years</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#12 Refactor doGetBeanNamesForType for improved readability and performance;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#10 35626: defaultCandidate for scoped proxies;#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#7 Add RSocketServiceMethod support for Kotlin suspending functions;#6 Add QUERY HTTP method;#4 Optimize parameter matching in TableMetaDataContext;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#4 Optimize parameter matching in TableMetaDataContext </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#12 Refactor doGetBeanNamesForType for improved readability and performance</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Risk Chart Overview
+ -&gt; La phrase en un texte, utiliser une visualisation pour ces 3 métriques</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">1 to 3 years</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#4 Optimize parameter matching in TableMetaDataContext;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#12 Refactor doGetBeanNamesForType for improved readability and performance;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#6 Add QUERY HTTP method;#7 Add RSocketServiceMethod support for Kotlin suspending functions;#10 35626: defaultCandidate for scoped proxies;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#10 35626: defaultCandidate for scoped proxies</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#4 Optimize parameter matching in TableMetaDataContext;#10 35626: defaultCandidate for scoped proxies;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#7 Add RSocketServiceMethod support for Kotlin suspending functions;#12 Refactor doGetBeanNamesForType for improved readability and performance;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#6 Add QUERY HTTP method;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#12 Refactor doGetBeanNamesForType for improved readability and performance;#10 35626: defaultCandidate for scoped proxies;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#4 Optimize parameter matching in TableMetaDataContext;#6 Add QUERY HTTP method;#7 Add RSocketServiceMethod support for Kotlin suspending functions;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">readability</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">lack of dimensions (of pr difficulties)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Spec coverage</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">NA</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">More dimensions</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">have a nice day</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#4 Optimize parameter matching in TableMetaDataContext;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#6 Add QUERY HTTP method;#10 35626: defaultCandidate for scoped proxies;#12 Refactor doGetBeanNamesForType for improved readability and performance;#7 Add RSocketServiceMethod support for Kotlin suspending functions;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Strongly disagree</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Quick impression of what the PR is like</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Not completely accurate for subtle difficulty</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Lines count;</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Friendlier explanation of the criteria</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">#4 Optimize parameter matching in TableMetaDataContext;#5 SingletonSupplier is not singleton if null is returned on first supplier call ;#10 35626: defaultCandidate for scoped proxies;#9 Release data buffer in AbstractCharSequenceDecoder even when String creation fails;#12 Refactor doGetBeanNamesForType for improved readability and performance;#3 Prevent NoClassDefFoundError when Jetty Reactive HttpClient is not available;#2 Normalize JAR entry paths to strip BOOT-INF/classes prefix in Spring-Boot fat JARs;#6 Add QUERY HTTP method;#7 Add RSocketServiceMethod support for Kotlin suspending functions;</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -808,8 +944,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:GU2" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:GU2"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:GU10" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:GU10"/>
   <x:tableColumns count="203">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Heure de début" dataDxfId="3"/>
@@ -2454,11 +2590,2547 @@
       <x:c r="GT2" s="10" t="s"/>
       <x:c r="GU2"/>
     </x:row>
+    <x:row r="3" hidden="0">
+      <x:c r="A3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="2">
+        <x:v>45957.7263541667</x:v>
+      </x:c>
+      <x:c r="C3" s="2">
+        <x:v>45957.7649074074</x:v>
+      </x:c>
+      <x:c r="D3" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E3" s="10" t="s"/>
+      <x:c r="F3"/>
+      <x:c r="G3" s="10" t="s"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J3"/>
+      <x:c r="K3" s="10" t="s"/>
+      <x:c r="L3" s="10" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="M3"/>
+      <x:c r="N3" s="10" t="s"/>
+      <x:c r="O3">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P3"/>
+      <x:c r="Q3" s="10" t="s"/>
+      <x:c r="R3" s="10" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="S3"/>
+      <x:c r="T3" s="10" t="s"/>
+      <x:c r="U3"/>
+      <x:c r="V3" s="10" t="s"/>
+      <x:c r="W3" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="X3"/>
+      <x:c r="Y3" s="10" t="s"/>
+      <x:c r="Z3" s="10" t="s"/>
+      <x:c r="AA3"/>
+      <x:c r="AB3" s="10" t="s"/>
+      <x:c r="AC3"/>
+      <x:c r="AD3" s="10" t="s"/>
+      <x:c r="AE3" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AF3" s="10" t="s"/>
+      <x:c r="AG3"/>
+      <x:c r="AH3" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AI3" s="10" t="s"/>
+      <x:c r="AJ3"/>
+      <x:c r="AK3" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AL3" s="10" t="s"/>
+      <x:c r="AM3"/>
+      <x:c r="AN3" s="10" t="s"/>
+      <x:c r="AO3" s="10" t="s"/>
+      <x:c r="AP3"/>
+      <x:c r="AQ3" s="10" t="s"/>
+      <x:c r="AR3" s="10" t="s"/>
+      <x:c r="AS3"/>
+      <x:c r="AT3" s="10" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="AU3" s="10" t="s"/>
+      <x:c r="AV3"/>
+      <x:c r="AW3" s="10" t="s"/>
+      <x:c r="AX3"/>
+      <x:c r="AY3" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AZ3" s="10" t="s"/>
+      <x:c r="BA3"/>
+      <x:c r="BB3" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC3"/>
+      <x:c r="BD3" s="10" t="s"/>
+      <x:c r="BE3" s="10" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="BF3"/>
+      <x:c r="BG3" s="10" t="s"/>
+      <x:c r="BH3"/>
+      <x:c r="BI3" s="10" t="s"/>
+      <x:c r="BJ3" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BK3"/>
+      <x:c r="BL3" s="10" t="s"/>
+      <x:c r="BM3" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BN3"/>
+      <x:c r="BO3" s="10" t="s"/>
+      <x:c r="BP3"/>
+      <x:c r="BQ3" s="10" t="s"/>
+      <x:c r="BR3" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BS3"/>
+      <x:c r="BT3" s="10" t="s"/>
+      <x:c r="BU3" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="BV3"/>
+      <x:c r="BW3" s="10" t="s"/>
+      <x:c r="BX3"/>
+      <x:c r="BY3" s="10" t="s"/>
+      <x:c r="BZ3" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA3"/>
+      <x:c r="CB3" s="10" t="s"/>
+      <x:c r="CC3" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="CD3"/>
+      <x:c r="CE3" s="10" t="s"/>
+      <x:c r="CF3" s="10" t="s"/>
+      <x:c r="CG3"/>
+      <x:c r="CH3" s="10" t="s"/>
+      <x:c r="CI3">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="CJ3"/>
+      <x:c r="CK3" s="10" t="s"/>
+      <x:c r="CL3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CM3"/>
+      <x:c r="CN3" s="10" t="s"/>
+      <x:c r="CO3">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CP3"/>
+      <x:c r="CQ3" s="10" t="s"/>
+      <x:c r="CR3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CS3"/>
+      <x:c r="CT3" s="10" t="s"/>
+      <x:c r="CU3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CV3"/>
+      <x:c r="CW3" s="10" t="s"/>
+      <x:c r="CX3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CY3" s="10" t="s"/>
+      <x:c r="CZ3"/>
+      <x:c r="DA3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DB3" s="10" t="s"/>
+      <x:c r="DC3"/>
+      <x:c r="DD3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DE3" s="10" t="s"/>
+      <x:c r="DF3"/>
+      <x:c r="DG3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DH3" s="10" t="s"/>
+      <x:c r="DI3"/>
+      <x:c r="DJ3">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DK3" s="10" t="s"/>
+      <x:c r="DL3"/>
+      <x:c r="DM3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DN3" s="10" t="s"/>
+      <x:c r="DO3"/>
+      <x:c r="DP3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DQ3" s="10" t="s"/>
+      <x:c r="DR3"/>
+      <x:c r="DS3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DT3" s="10" t="s"/>
+      <x:c r="DU3"/>
+      <x:c r="DV3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DW3" s="10" t="s"/>
+      <x:c r="DX3"/>
+      <x:c r="DY3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DZ3" s="10" t="s"/>
+      <x:c r="EA3"/>
+      <x:c r="EB3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC3" s="10" t="s"/>
+      <x:c r="ED3"/>
+      <x:c r="EE3">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EF3" s="10" t="s"/>
+      <x:c r="EG3"/>
+      <x:c r="EH3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EI3" s="10" t="s"/>
+      <x:c r="EJ3"/>
+      <x:c r="EK3">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EL3" s="10" t="s"/>
+      <x:c r="EM3"/>
+      <x:c r="EN3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EO3" s="10" t="s"/>
+      <x:c r="EP3"/>
+      <x:c r="EQ3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="ER3" s="10" t="s"/>
+      <x:c r="ES3"/>
+      <x:c r="ET3">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EU3" s="10" t="s"/>
+      <x:c r="EV3"/>
+      <x:c r="EW3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EX3" s="10" t="s"/>
+      <x:c r="EY3"/>
+      <x:c r="EZ3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FA3" s="10" t="s"/>
+      <x:c r="FB3"/>
+      <x:c r="FC3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FD3" s="10" t="s"/>
+      <x:c r="FE3"/>
+      <x:c r="FF3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FG3" s="10" t="s"/>
+      <x:c r="FH3"/>
+      <x:c r="FI3">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FJ3" s="10" t="s"/>
+      <x:c r="FK3"/>
+      <x:c r="FL3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FM3" s="10" t="s"/>
+      <x:c r="FN3"/>
+      <x:c r="FO3">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FP3" s="10" t="s"/>
+      <x:c r="FQ3"/>
+      <x:c r="FR3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FS3" s="10" t="s"/>
+      <x:c r="FT3"/>
+      <x:c r="FU3">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FV3" s="10" t="s"/>
+      <x:c r="FW3"/>
+      <x:c r="FX3" s="10" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="FY3" s="10" t="s"/>
+      <x:c r="FZ3"/>
+      <x:c r="GA3" s="10" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="GB3" s="10" t="s"/>
+      <x:c r="GC3"/>
+      <x:c r="GD3" s="10" t="s"/>
+      <x:c r="GE3" s="10" t="s"/>
+      <x:c r="GF3"/>
+      <x:c r="GG3" s="10" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="GH3" s="10" t="s"/>
+      <x:c r="GI3"/>
+      <x:c r="GJ3" s="10" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="GK3" s="10" t="s"/>
+      <x:c r="GL3"/>
+      <x:c r="GM3" s="10" t="s"/>
+      <x:c r="GN3" s="10" t="s"/>
+      <x:c r="GO3"/>
+      <x:c r="GP3" s="10" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="GQ3" s="10" t="s"/>
+      <x:c r="GR3"/>
+      <x:c r="GS3" s="10" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="GT3" s="10" t="s"/>
+      <x:c r="GU3"/>
+    </x:row>
+    <x:row r="4" hidden="0">
+      <x:c r="A4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="2">
+        <x:v>45959.3805902778</x:v>
+      </x:c>
+      <x:c r="C4" s="2">
+        <x:v>45959.4203009259</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="s"/>
+      <x:c r="F4"/>
+      <x:c r="G4" s="10" t="s"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J4"/>
+      <x:c r="K4" s="10" t="s"/>
+      <x:c r="L4" s="10" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="M4"/>
+      <x:c r="N4" s="10" t="s"/>
+      <x:c r="O4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P4"/>
+      <x:c r="Q4" s="10" t="s"/>
+      <x:c r="R4" s="10" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="S4"/>
+      <x:c r="T4" s="10" t="s"/>
+      <x:c r="U4"/>
+      <x:c r="V4" s="10" t="s"/>
+      <x:c r="W4" s="10" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="X4"/>
+      <x:c r="Y4" s="10" t="s"/>
+      <x:c r="Z4" s="10" t="s"/>
+      <x:c r="AA4"/>
+      <x:c r="AB4" s="10" t="s"/>
+      <x:c r="AC4"/>
+      <x:c r="AD4" s="10" t="s"/>
+      <x:c r="AE4" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AF4" s="10" t="s"/>
+      <x:c r="AG4"/>
+      <x:c r="AH4" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AI4" s="10" t="s"/>
+      <x:c r="AJ4"/>
+      <x:c r="AK4" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AL4" s="10" t="s"/>
+      <x:c r="AM4"/>
+      <x:c r="AN4" s="10" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="AO4" s="10" t="s"/>
+      <x:c r="AP4"/>
+      <x:c r="AQ4" s="10" t="s"/>
+      <x:c r="AR4" s="10" t="s"/>
+      <x:c r="AS4"/>
+      <x:c r="AT4" s="10" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="AU4" s="10" t="s"/>
+      <x:c r="AV4"/>
+      <x:c r="AW4" s="10" t="s"/>
+      <x:c r="AX4"/>
+      <x:c r="AY4" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="AZ4" s="10" t="s"/>
+      <x:c r="BA4"/>
+      <x:c r="BB4" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC4"/>
+      <x:c r="BD4" s="10" t="s"/>
+      <x:c r="BE4" s="10" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="BF4"/>
+      <x:c r="BG4" s="10" t="s"/>
+      <x:c r="BH4"/>
+      <x:c r="BI4" s="10" t="s"/>
+      <x:c r="BJ4" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BK4"/>
+      <x:c r="BL4" s="10" t="s"/>
+      <x:c r="BM4" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="BN4"/>
+      <x:c r="BO4" s="10" t="s"/>
+      <x:c r="BP4"/>
+      <x:c r="BQ4" s="10" t="s"/>
+      <x:c r="BR4" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BS4"/>
+      <x:c r="BT4" s="10" t="s"/>
+      <x:c r="BU4" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BV4"/>
+      <x:c r="BW4" s="10" t="s"/>
+      <x:c r="BX4"/>
+      <x:c r="BY4" s="10" t="s"/>
+      <x:c r="BZ4" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA4"/>
+      <x:c r="CB4" s="10" t="s"/>
+      <x:c r="CC4" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="CD4"/>
+      <x:c r="CE4" s="10" t="s"/>
+      <x:c r="CF4" s="10" t="s"/>
+      <x:c r="CG4"/>
+      <x:c r="CH4" s="10" t="s"/>
+      <x:c r="CI4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CJ4"/>
+      <x:c r="CK4" s="10" t="s"/>
+      <x:c r="CL4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CM4"/>
+      <x:c r="CN4" s="10" t="s"/>
+      <x:c r="CO4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CP4"/>
+      <x:c r="CQ4" s="10" t="s"/>
+      <x:c r="CR4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS4"/>
+      <x:c r="CT4" s="10" t="s"/>
+      <x:c r="CU4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CV4"/>
+      <x:c r="CW4" s="10" t="s"/>
+      <x:c r="CX4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CY4" s="10" t="s"/>
+      <x:c r="CZ4"/>
+      <x:c r="DA4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DB4" s="10" t="s"/>
+      <x:c r="DC4"/>
+      <x:c r="DD4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DE4" s="10" t="s"/>
+      <x:c r="DF4"/>
+      <x:c r="DG4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DH4" s="10" t="s"/>
+      <x:c r="DI4"/>
+      <x:c r="DJ4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DK4" s="10" t="s"/>
+      <x:c r="DL4"/>
+      <x:c r="DM4">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DN4" s="10" t="s"/>
+      <x:c r="DO4"/>
+      <x:c r="DP4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DQ4" s="10" t="s"/>
+      <x:c r="DR4"/>
+      <x:c r="DS4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DT4" s="10" t="s"/>
+      <x:c r="DU4"/>
+      <x:c r="DV4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DW4" s="10" t="s"/>
+      <x:c r="DX4"/>
+      <x:c r="DY4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DZ4" s="10" t="s"/>
+      <x:c r="EA4"/>
+      <x:c r="EB4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC4" s="10" t="s"/>
+      <x:c r="ED4"/>
+      <x:c r="EE4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EF4" s="10" t="s"/>
+      <x:c r="EG4"/>
+      <x:c r="EH4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EI4" s="10" t="s"/>
+      <x:c r="EJ4"/>
+      <x:c r="EK4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EL4" s="10" t="s"/>
+      <x:c r="EM4"/>
+      <x:c r="EN4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EO4" s="10" t="s"/>
+      <x:c r="EP4"/>
+      <x:c r="EQ4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="ER4" s="10" t="s"/>
+      <x:c r="ES4"/>
+      <x:c r="ET4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EU4" s="10" t="s"/>
+      <x:c r="EV4"/>
+      <x:c r="EW4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EX4" s="10" t="s"/>
+      <x:c r="EY4"/>
+      <x:c r="EZ4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FA4" s="10" t="s"/>
+      <x:c r="FB4"/>
+      <x:c r="FC4">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FD4" s="10" t="s"/>
+      <x:c r="FE4"/>
+      <x:c r="FF4">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FG4" s="10" t="s"/>
+      <x:c r="FH4"/>
+      <x:c r="FI4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FJ4" s="10" t="s"/>
+      <x:c r="FK4"/>
+      <x:c r="FL4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FM4" s="10" t="s"/>
+      <x:c r="FN4"/>
+      <x:c r="FO4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FP4" s="10" t="s"/>
+      <x:c r="FQ4"/>
+      <x:c r="FR4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS4" s="10" t="s"/>
+      <x:c r="FT4"/>
+      <x:c r="FU4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FV4" s="10" t="s"/>
+      <x:c r="FW4"/>
+      <x:c r="FX4" s="10" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="FY4" s="10" t="s"/>
+      <x:c r="FZ4"/>
+      <x:c r="GA4" s="10" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="GB4" s="10" t="s"/>
+      <x:c r="GC4"/>
+      <x:c r="GD4" s="10" t="s"/>
+      <x:c r="GE4" s="10" t="s"/>
+      <x:c r="GF4"/>
+      <x:c r="GG4" s="10" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="GH4" s="10" t="s"/>
+      <x:c r="GI4"/>
+      <x:c r="GJ4" s="10" t="s"/>
+      <x:c r="GK4" s="10" t="s"/>
+      <x:c r="GL4"/>
+      <x:c r="GM4" s="10" t="s">
+        <x:v>236</x:v>
+      </x:c>
+      <x:c r="GN4" s="10" t="s"/>
+      <x:c r="GO4"/>
+      <x:c r="GP4" s="10" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="GQ4" s="10" t="s"/>
+      <x:c r="GR4"/>
+      <x:c r="GS4" s="10" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="GT4" s="10" t="s"/>
+      <x:c r="GU4"/>
+    </x:row>
+    <x:row r="5" hidden="0">
+      <x:c r="A5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="2">
+        <x:v>45959.4270023148</x:v>
+      </x:c>
+      <x:c r="C5" s="2">
+        <x:v>45959.4684606481</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E5" s="10" t="s"/>
+      <x:c r="F5"/>
+      <x:c r="G5" s="10" t="s"/>
+      <x:c r="H5" s="2"/>
+      <x:c r="I5" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J5"/>
+      <x:c r="K5" s="10" t="s"/>
+      <x:c r="L5" s="10" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="M5"/>
+      <x:c r="N5" s="10" t="s"/>
+      <x:c r="O5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P5"/>
+      <x:c r="Q5" s="10" t="s"/>
+      <x:c r="R5" s="10" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="S5"/>
+      <x:c r="T5" s="10" t="s"/>
+      <x:c r="U5"/>
+      <x:c r="V5" s="10" t="s"/>
+      <x:c r="W5" s="10" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="X5"/>
+      <x:c r="Y5" s="10" t="s"/>
+      <x:c r="Z5" s="10" t="s"/>
+      <x:c r="AA5"/>
+      <x:c r="AB5" s="10" t="s"/>
+      <x:c r="AC5"/>
+      <x:c r="AD5" s="10" t="s"/>
+      <x:c r="AE5" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AF5" s="10" t="s"/>
+      <x:c r="AG5"/>
+      <x:c r="AH5" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="AI5" s="10" t="s"/>
+      <x:c r="AJ5"/>
+      <x:c r="AK5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AL5" s="10" t="s"/>
+      <x:c r="AM5"/>
+      <x:c r="AN5" s="10" t="s"/>
+      <x:c r="AO5" s="10" t="s"/>
+      <x:c r="AP5"/>
+      <x:c r="AQ5" s="10" t="s"/>
+      <x:c r="AR5" s="10" t="s"/>
+      <x:c r="AS5"/>
+      <x:c r="AT5" s="10" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="AU5" s="10" t="s"/>
+      <x:c r="AV5"/>
+      <x:c r="AW5" s="10" t="s"/>
+      <x:c r="AX5"/>
+      <x:c r="AY5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AZ5" s="10" t="s"/>
+      <x:c r="BA5"/>
+      <x:c r="BB5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC5"/>
+      <x:c r="BD5" s="10" t="s"/>
+      <x:c r="BE5" s="10" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="BF5"/>
+      <x:c r="BG5" s="10" t="s"/>
+      <x:c r="BH5"/>
+      <x:c r="BI5" s="10" t="s"/>
+      <x:c r="BJ5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BK5"/>
+      <x:c r="BL5" s="10" t="s"/>
+      <x:c r="BM5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BN5"/>
+      <x:c r="BO5" s="10" t="s"/>
+      <x:c r="BP5"/>
+      <x:c r="BQ5" s="10" t="s"/>
+      <x:c r="BR5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BS5"/>
+      <x:c r="BT5" s="10" t="s"/>
+      <x:c r="BU5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BV5"/>
+      <x:c r="BW5" s="10" t="s"/>
+      <x:c r="BX5"/>
+      <x:c r="BY5" s="10" t="s"/>
+      <x:c r="BZ5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="CA5"/>
+      <x:c r="CB5" s="10" t="s"/>
+      <x:c r="CC5" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="CD5"/>
+      <x:c r="CE5" s="10" t="s"/>
+      <x:c r="CF5" s="10" t="s"/>
+      <x:c r="CG5"/>
+      <x:c r="CH5" s="10" t="s"/>
+      <x:c r="CI5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="CJ5"/>
+      <x:c r="CK5" s="10" t="s"/>
+      <x:c r="CL5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CM5"/>
+      <x:c r="CN5" s="10" t="s"/>
+      <x:c r="CO5">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CP5"/>
+      <x:c r="CQ5" s="10" t="s"/>
+      <x:c r="CR5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS5"/>
+      <x:c r="CT5" s="10" t="s"/>
+      <x:c r="CU5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV5"/>
+      <x:c r="CW5" s="10" t="s"/>
+      <x:c r="CX5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CY5" s="10" t="s"/>
+      <x:c r="CZ5"/>
+      <x:c r="DA5">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DB5" s="10" t="s"/>
+      <x:c r="DC5"/>
+      <x:c r="DD5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DE5" s="10" t="s"/>
+      <x:c r="DF5"/>
+      <x:c r="DG5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DH5" s="10" t="s"/>
+      <x:c r="DI5"/>
+      <x:c r="DJ5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DK5" s="10" t="s"/>
+      <x:c r="DL5"/>
+      <x:c r="DM5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DN5" s="10" t="s"/>
+      <x:c r="DO5"/>
+      <x:c r="DP5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="DQ5" s="10" t="s"/>
+      <x:c r="DR5"/>
+      <x:c r="DS5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DT5" s="10" t="s"/>
+      <x:c r="DU5"/>
+      <x:c r="DV5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DW5" s="10" t="s"/>
+      <x:c r="DX5"/>
+      <x:c r="DY5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DZ5" s="10" t="s"/>
+      <x:c r="EA5"/>
+      <x:c r="EB5">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC5" s="10" t="s"/>
+      <x:c r="ED5"/>
+      <x:c r="EE5">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EF5" s="10" t="s"/>
+      <x:c r="EG5"/>
+      <x:c r="EH5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EI5" s="10" t="s"/>
+      <x:c r="EJ5"/>
+      <x:c r="EK5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EL5" s="10" t="s"/>
+      <x:c r="EM5"/>
+      <x:c r="EN5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="EO5" s="10" t="s"/>
+      <x:c r="EP5"/>
+      <x:c r="EQ5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="ER5" s="10" t="s"/>
+      <x:c r="ES5"/>
+      <x:c r="ET5">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="EU5" s="10" t="s"/>
+      <x:c r="EV5"/>
+      <x:c r="EW5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EX5" s="10" t="s"/>
+      <x:c r="EY5"/>
+      <x:c r="EZ5">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FA5" s="10" t="s"/>
+      <x:c r="FB5"/>
+      <x:c r="FC5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FD5" s="10" t="s"/>
+      <x:c r="FE5"/>
+      <x:c r="FF5">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="FG5" s="10" t="s"/>
+      <x:c r="FH5"/>
+      <x:c r="FI5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FJ5" s="10" t="s"/>
+      <x:c r="FK5"/>
+      <x:c r="FL5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FM5" s="10" t="s"/>
+      <x:c r="FN5"/>
+      <x:c r="FO5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FP5" s="10" t="s"/>
+      <x:c r="FQ5"/>
+      <x:c r="FR5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS5" s="10" t="s"/>
+      <x:c r="FT5"/>
+      <x:c r="FU5">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FV5" s="10" t="s"/>
+      <x:c r="FW5"/>
+      <x:c r="FX5" s="10" t="s"/>
+      <x:c r="FY5" s="10" t="s"/>
+      <x:c r="FZ5"/>
+      <x:c r="GA5" s="10" t="s"/>
+      <x:c r="GB5" s="10" t="s"/>
+      <x:c r="GC5"/>
+      <x:c r="GD5" s="10" t="s"/>
+      <x:c r="GE5" s="10" t="s"/>
+      <x:c r="GF5"/>
+      <x:c r="GG5" s="10" t="s"/>
+      <x:c r="GH5" s="10" t="s"/>
+      <x:c r="GI5"/>
+      <x:c r="GJ5" s="10" t="s"/>
+      <x:c r="GK5" s="10" t="s"/>
+      <x:c r="GL5"/>
+      <x:c r="GM5" s="10" t="s"/>
+      <x:c r="GN5" s="10" t="s"/>
+      <x:c r="GO5"/>
+      <x:c r="GP5" s="10" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="GQ5" s="10" t="s"/>
+      <x:c r="GR5"/>
+      <x:c r="GS5" s="10" t="s"/>
+      <x:c r="GT5" s="10" t="s"/>
+      <x:c r="GU5"/>
+    </x:row>
+    <x:row r="6" hidden="0">
+      <x:c r="A6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="2">
+        <x:v>45959.5470023148</x:v>
+      </x:c>
+      <x:c r="C6" s="2">
+        <x:v>45959.5877083333</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="s"/>
+      <x:c r="F6"/>
+      <x:c r="G6" s="10" t="s"/>
+      <x:c r="H6" s="2"/>
+      <x:c r="I6" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J6"/>
+      <x:c r="K6" s="10" t="s"/>
+      <x:c r="L6" s="10" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="M6"/>
+      <x:c r="N6" s="10" t="s"/>
+      <x:c r="O6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P6"/>
+      <x:c r="Q6" s="10" t="s"/>
+      <x:c r="R6" s="10" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="S6"/>
+      <x:c r="T6" s="10" t="s"/>
+      <x:c r="U6"/>
+      <x:c r="V6" s="10" t="s"/>
+      <x:c r="W6" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="X6"/>
+      <x:c r="Y6" s="10" t="s"/>
+      <x:c r="Z6" s="10" t="s"/>
+      <x:c r="AA6"/>
+      <x:c r="AB6" s="10" t="s"/>
+      <x:c r="AC6"/>
+      <x:c r="AD6" s="10" t="s"/>
+      <x:c r="AE6" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AF6" s="10" t="s"/>
+      <x:c r="AG6"/>
+      <x:c r="AH6" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AI6" s="10" t="s"/>
+      <x:c r="AJ6"/>
+      <x:c r="AK6" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AL6" s="10" t="s"/>
+      <x:c r="AM6"/>
+      <x:c r="AN6" s="10" t="s"/>
+      <x:c r="AO6" s="10" t="s"/>
+      <x:c r="AP6"/>
+      <x:c r="AQ6" s="10" t="s"/>
+      <x:c r="AR6" s="10" t="s"/>
+      <x:c r="AS6"/>
+      <x:c r="AT6" s="10" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="AU6" s="10" t="s"/>
+      <x:c r="AV6"/>
+      <x:c r="AW6" s="10" t="s"/>
+      <x:c r="AX6"/>
+      <x:c r="AY6" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AZ6" s="10" t="s"/>
+      <x:c r="BA6"/>
+      <x:c r="BB6" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="BC6"/>
+      <x:c r="BD6" s="10" t="s"/>
+      <x:c r="BE6" s="10" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="BF6"/>
+      <x:c r="BG6" s="10" t="s"/>
+      <x:c r="BH6"/>
+      <x:c r="BI6" s="10" t="s"/>
+      <x:c r="BJ6" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BK6"/>
+      <x:c r="BL6" s="10" t="s"/>
+      <x:c r="BM6" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="BN6"/>
+      <x:c r="BO6" s="10" t="s"/>
+      <x:c r="BP6"/>
+      <x:c r="BQ6" s="10" t="s"/>
+      <x:c r="BR6" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BS6"/>
+      <x:c r="BT6" s="10" t="s"/>
+      <x:c r="BU6" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="BV6"/>
+      <x:c r="BW6" s="10" t="s"/>
+      <x:c r="BX6"/>
+      <x:c r="BY6" s="10" t="s"/>
+      <x:c r="BZ6" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA6"/>
+      <x:c r="CB6" s="10" t="s"/>
+      <x:c r="CC6" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CD6"/>
+      <x:c r="CE6" s="10" t="s"/>
+      <x:c r="CF6" s="10" t="s"/>
+      <x:c r="CG6"/>
+      <x:c r="CH6" s="10" t="s"/>
+      <x:c r="CI6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CJ6"/>
+      <x:c r="CK6" s="10" t="s"/>
+      <x:c r="CL6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CM6"/>
+      <x:c r="CN6" s="10" t="s"/>
+      <x:c r="CO6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CP6"/>
+      <x:c r="CQ6" s="10" t="s"/>
+      <x:c r="CR6">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS6"/>
+      <x:c r="CT6" s="10" t="s"/>
+      <x:c r="CU6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CV6"/>
+      <x:c r="CW6" s="10" t="s"/>
+      <x:c r="CX6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CY6" s="10" t="s"/>
+      <x:c r="CZ6"/>
+      <x:c r="DA6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DB6" s="10" t="s"/>
+      <x:c r="DC6"/>
+      <x:c r="DD6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DE6" s="10" t="s"/>
+      <x:c r="DF6"/>
+      <x:c r="DG6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DH6" s="10" t="s"/>
+      <x:c r="DI6"/>
+      <x:c r="DJ6">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DK6" s="10" t="s"/>
+      <x:c r="DL6"/>
+      <x:c r="DM6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DN6" s="10" t="s"/>
+      <x:c r="DO6"/>
+      <x:c r="DP6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DQ6" s="10" t="s"/>
+      <x:c r="DR6"/>
+      <x:c r="DS6">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DT6" s="10" t="s"/>
+      <x:c r="DU6"/>
+      <x:c r="DV6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DW6" s="10" t="s"/>
+      <x:c r="DX6"/>
+      <x:c r="DY6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DZ6" s="10" t="s"/>
+      <x:c r="EA6"/>
+      <x:c r="EB6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EC6" s="10" t="s"/>
+      <x:c r="ED6"/>
+      <x:c r="EE6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EF6" s="10" t="s"/>
+      <x:c r="EG6"/>
+      <x:c r="EH6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EI6" s="10" t="s"/>
+      <x:c r="EJ6"/>
+      <x:c r="EK6">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EL6" s="10" t="s"/>
+      <x:c r="EM6"/>
+      <x:c r="EN6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EO6" s="10" t="s"/>
+      <x:c r="EP6"/>
+      <x:c r="EQ6">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="ER6" s="10" t="s"/>
+      <x:c r="ES6"/>
+      <x:c r="ET6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EU6" s="10" t="s"/>
+      <x:c r="EV6"/>
+      <x:c r="EW6">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EX6" s="10" t="s"/>
+      <x:c r="EY6"/>
+      <x:c r="EZ6">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FA6" s="10" t="s"/>
+      <x:c r="FB6"/>
+      <x:c r="FC6">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FD6" s="10" t="s"/>
+      <x:c r="FE6"/>
+      <x:c r="FF6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FG6" s="10" t="s"/>
+      <x:c r="FH6"/>
+      <x:c r="FI6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FJ6" s="10" t="s"/>
+      <x:c r="FK6"/>
+      <x:c r="FL6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FM6" s="10" t="s"/>
+      <x:c r="FN6"/>
+      <x:c r="FO6">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FP6" s="10" t="s"/>
+      <x:c r="FQ6"/>
+      <x:c r="FR6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS6" s="10" t="s"/>
+      <x:c r="FT6"/>
+      <x:c r="FU6">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FV6" s="10" t="s"/>
+      <x:c r="FW6"/>
+      <x:c r="FX6" s="10" t="s"/>
+      <x:c r="FY6" s="10" t="s"/>
+      <x:c r="FZ6"/>
+      <x:c r="GA6" s="10" t="s"/>
+      <x:c r="GB6" s="10" t="s"/>
+      <x:c r="GC6"/>
+      <x:c r="GD6" s="10" t="s"/>
+      <x:c r="GE6" s="10" t="s"/>
+      <x:c r="GF6"/>
+      <x:c r="GG6" s="10" t="s"/>
+      <x:c r="GH6" s="10" t="s"/>
+      <x:c r="GI6"/>
+      <x:c r="GJ6" s="10" t="s"/>
+      <x:c r="GK6" s="10" t="s"/>
+      <x:c r="GL6"/>
+      <x:c r="GM6" s="10" t="s"/>
+      <x:c r="GN6" s="10" t="s"/>
+      <x:c r="GO6"/>
+      <x:c r="GP6" s="10" t="s"/>
+      <x:c r="GQ6" s="10" t="s"/>
+      <x:c r="GR6"/>
+      <x:c r="GS6" s="10" t="s"/>
+      <x:c r="GT6" s="10" t="s"/>
+      <x:c r="GU6"/>
+    </x:row>
+    <x:row r="7" hidden="0">
+      <x:c r="A7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="2">
+        <x:v>45959.5932638889</x:v>
+      </x:c>
+      <x:c r="C7" s="2">
+        <x:v>45959.6342361111</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="s"/>
+      <x:c r="F7"/>
+      <x:c r="G7" s="10" t="s"/>
+      <x:c r="H7" s="2"/>
+      <x:c r="I7" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J7"/>
+      <x:c r="K7" s="10" t="s"/>
+      <x:c r="L7" s="10" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="M7"/>
+      <x:c r="N7" s="10" t="s"/>
+      <x:c r="O7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P7"/>
+      <x:c r="Q7" s="10" t="s"/>
+      <x:c r="R7" s="10" t="s">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="S7"/>
+      <x:c r="T7" s="10" t="s"/>
+      <x:c r="U7"/>
+      <x:c r="V7" s="10" t="s"/>
+      <x:c r="W7" s="10" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="X7"/>
+      <x:c r="Y7" s="10" t="s"/>
+      <x:c r="Z7" s="10" t="s"/>
+      <x:c r="AA7"/>
+      <x:c r="AB7" s="10" t="s"/>
+      <x:c r="AC7"/>
+      <x:c r="AD7" s="10" t="s"/>
+      <x:c r="AE7" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AF7" s="10" t="s"/>
+      <x:c r="AG7"/>
+      <x:c r="AH7" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AI7" s="10" t="s"/>
+      <x:c r="AJ7"/>
+      <x:c r="AK7" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AL7" s="10" t="s"/>
+      <x:c r="AM7"/>
+      <x:c r="AN7" s="10" t="s"/>
+      <x:c r="AO7" s="10" t="s"/>
+      <x:c r="AP7"/>
+      <x:c r="AQ7" s="10" t="s"/>
+      <x:c r="AR7" s="10" t="s"/>
+      <x:c r="AS7"/>
+      <x:c r="AT7" s="10" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="AU7" s="10" t="s"/>
+      <x:c r="AV7"/>
+      <x:c r="AW7" s="10" t="s"/>
+      <x:c r="AX7"/>
+      <x:c r="AY7" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="AZ7" s="10" t="s"/>
+      <x:c r="BA7"/>
+      <x:c r="BB7" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC7"/>
+      <x:c r="BD7" s="10" t="s"/>
+      <x:c r="BE7" s="10" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="BF7"/>
+      <x:c r="BG7" s="10" t="s"/>
+      <x:c r="BH7"/>
+      <x:c r="BI7" s="10" t="s"/>
+      <x:c r="BJ7" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BK7"/>
+      <x:c r="BL7" s="10" t="s"/>
+      <x:c r="BM7" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BN7"/>
+      <x:c r="BO7" s="10" t="s"/>
+      <x:c r="BP7"/>
+      <x:c r="BQ7" s="10" t="s"/>
+      <x:c r="BR7" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BS7"/>
+      <x:c r="BT7" s="10" t="s"/>
+      <x:c r="BU7" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BV7"/>
+      <x:c r="BW7" s="10" t="s"/>
+      <x:c r="BX7"/>
+      <x:c r="BY7" s="10" t="s"/>
+      <x:c r="BZ7" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA7"/>
+      <x:c r="CB7" s="10" t="s"/>
+      <x:c r="CC7" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CD7"/>
+      <x:c r="CE7" s="10" t="s"/>
+      <x:c r="CF7" s="10" t="s"/>
+      <x:c r="CG7"/>
+      <x:c r="CH7" s="10" t="s"/>
+      <x:c r="CI7">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="CJ7"/>
+      <x:c r="CK7" s="10" t="s"/>
+      <x:c r="CL7">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CM7"/>
+      <x:c r="CN7" s="10" t="s"/>
+      <x:c r="CO7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CP7"/>
+      <x:c r="CQ7" s="10" t="s"/>
+      <x:c r="CR7">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CS7"/>
+      <x:c r="CT7" s="10" t="s"/>
+      <x:c r="CU7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CV7"/>
+      <x:c r="CW7" s="10" t="s"/>
+      <x:c r="CX7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CY7" s="10" t="s"/>
+      <x:c r="CZ7"/>
+      <x:c r="DA7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DB7" s="10" t="s"/>
+      <x:c r="DC7"/>
+      <x:c r="DD7">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DE7" s="10" t="s"/>
+      <x:c r="DF7"/>
+      <x:c r="DG7">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="DH7" s="10" t="s"/>
+      <x:c r="DI7"/>
+      <x:c r="DJ7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DK7" s="10" t="s"/>
+      <x:c r="DL7"/>
+      <x:c r="DM7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DN7" s="10" t="s"/>
+      <x:c r="DO7"/>
+      <x:c r="DP7">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="DQ7" s="10" t="s"/>
+      <x:c r="DR7"/>
+      <x:c r="DS7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DT7" s="10" t="s"/>
+      <x:c r="DU7"/>
+      <x:c r="DV7">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DW7" s="10" t="s"/>
+      <x:c r="DX7"/>
+      <x:c r="DY7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DZ7" s="10" t="s"/>
+      <x:c r="EA7"/>
+      <x:c r="EB7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC7" s="10" t="s"/>
+      <x:c r="ED7"/>
+      <x:c r="EE7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EF7" s="10" t="s"/>
+      <x:c r="EG7"/>
+      <x:c r="EH7">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EI7" s="10" t="s"/>
+      <x:c r="EJ7"/>
+      <x:c r="EK7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EL7" s="10" t="s"/>
+      <x:c r="EM7"/>
+      <x:c r="EN7">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EO7" s="10" t="s"/>
+      <x:c r="EP7"/>
+      <x:c r="EQ7">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="ER7" s="10" t="s"/>
+      <x:c r="ES7"/>
+      <x:c r="ET7">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="EU7" s="10" t="s"/>
+      <x:c r="EV7"/>
+      <x:c r="EW7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EX7" s="10" t="s"/>
+      <x:c r="EY7"/>
+      <x:c r="EZ7">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FA7" s="10" t="s"/>
+      <x:c r="FB7"/>
+      <x:c r="FC7">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FD7" s="10" t="s"/>
+      <x:c r="FE7"/>
+      <x:c r="FF7">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="FG7" s="10" t="s"/>
+      <x:c r="FH7"/>
+      <x:c r="FI7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FJ7" s="10" t="s"/>
+      <x:c r="FK7"/>
+      <x:c r="FL7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FM7" s="10" t="s"/>
+      <x:c r="FN7"/>
+      <x:c r="FO7">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FP7" s="10" t="s"/>
+      <x:c r="FQ7"/>
+      <x:c r="FR7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS7" s="10" t="s"/>
+      <x:c r="FT7"/>
+      <x:c r="FU7">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FV7" s="10" t="s"/>
+      <x:c r="FW7"/>
+      <x:c r="FX7" s="10" t="s"/>
+      <x:c r="FY7" s="10" t="s"/>
+      <x:c r="FZ7"/>
+      <x:c r="GA7" s="10" t="s"/>
+      <x:c r="GB7" s="10" t="s"/>
+      <x:c r="GC7"/>
+      <x:c r="GD7" s="10" t="s"/>
+      <x:c r="GE7" s="10" t="s"/>
+      <x:c r="GF7"/>
+      <x:c r="GG7" s="10" t="s"/>
+      <x:c r="GH7" s="10" t="s"/>
+      <x:c r="GI7"/>
+      <x:c r="GJ7" s="10" t="s"/>
+      <x:c r="GK7" s="10" t="s"/>
+      <x:c r="GL7"/>
+      <x:c r="GM7" s="10" t="s"/>
+      <x:c r="GN7" s="10" t="s"/>
+      <x:c r="GO7"/>
+      <x:c r="GP7" s="10" t="s"/>
+      <x:c r="GQ7" s="10" t="s"/>
+      <x:c r="GR7"/>
+      <x:c r="GS7" s="10" t="s"/>
+      <x:c r="GT7" s="10" t="s"/>
+      <x:c r="GU7"/>
+    </x:row>
+    <x:row r="8" hidden="0">
+      <x:c r="A8">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="2">
+        <x:v>45959.6409837963</x:v>
+      </x:c>
+      <x:c r="C8" s="2">
+        <x:v>45959.6774884259</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="s"/>
+      <x:c r="F8"/>
+      <x:c r="G8" s="10" t="s"/>
+      <x:c r="H8" s="2"/>
+      <x:c r="I8" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J8"/>
+      <x:c r="K8" s="10" t="s"/>
+      <x:c r="L8" s="10" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="M8"/>
+      <x:c r="N8" s="10" t="s"/>
+      <x:c r="O8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P8"/>
+      <x:c r="Q8" s="10" t="s"/>
+      <x:c r="R8" s="10" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="S8"/>
+      <x:c r="T8" s="10" t="s"/>
+      <x:c r="U8"/>
+      <x:c r="V8" s="10" t="s"/>
+      <x:c r="W8" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="X8"/>
+      <x:c r="Y8" s="10" t="s"/>
+      <x:c r="Z8" s="10" t="s"/>
+      <x:c r="AA8"/>
+      <x:c r="AB8" s="10" t="s"/>
+      <x:c r="AC8"/>
+      <x:c r="AD8" s="10" t="s"/>
+      <x:c r="AE8" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AF8" s="10" t="s"/>
+      <x:c r="AG8"/>
+      <x:c r="AH8" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="AI8" s="10" t="s"/>
+      <x:c r="AJ8"/>
+      <x:c r="AK8" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AL8" s="10" t="s"/>
+      <x:c r="AM8"/>
+      <x:c r="AN8" s="10" t="s"/>
+      <x:c r="AO8" s="10" t="s"/>
+      <x:c r="AP8"/>
+      <x:c r="AQ8" s="10" t="s"/>
+      <x:c r="AR8" s="10" t="s"/>
+      <x:c r="AS8"/>
+      <x:c r="AT8" s="10" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="AU8" s="10" t="s"/>
+      <x:c r="AV8"/>
+      <x:c r="AW8" s="10" t="s"/>
+      <x:c r="AX8"/>
+      <x:c r="AY8" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AZ8" s="10" t="s"/>
+      <x:c r="BA8"/>
+      <x:c r="BB8" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC8"/>
+      <x:c r="BD8" s="10" t="s"/>
+      <x:c r="BE8" s="10" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="BF8"/>
+      <x:c r="BG8" s="10" t="s"/>
+      <x:c r="BH8"/>
+      <x:c r="BI8" s="10" t="s"/>
+      <x:c r="BJ8" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BK8"/>
+      <x:c r="BL8" s="10" t="s"/>
+      <x:c r="BM8" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="BN8"/>
+      <x:c r="BO8" s="10" t="s"/>
+      <x:c r="BP8"/>
+      <x:c r="BQ8" s="10" t="s"/>
+      <x:c r="BR8" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BS8"/>
+      <x:c r="BT8" s="10" t="s"/>
+      <x:c r="BU8" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BV8"/>
+      <x:c r="BW8" s="10" t="s"/>
+      <x:c r="BX8"/>
+      <x:c r="BY8" s="10" t="s"/>
+      <x:c r="BZ8" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="CA8"/>
+      <x:c r="CB8" s="10" t="s"/>
+      <x:c r="CC8" s="10" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="CD8"/>
+      <x:c r="CE8" s="10" t="s"/>
+      <x:c r="CF8" s="10" t="s"/>
+      <x:c r="CG8"/>
+      <x:c r="CH8" s="10" t="s"/>
+      <x:c r="CI8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CJ8"/>
+      <x:c r="CK8" s="10" t="s"/>
+      <x:c r="CL8">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CM8"/>
+      <x:c r="CN8" s="10" t="s"/>
+      <x:c r="CO8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CP8"/>
+      <x:c r="CQ8" s="10" t="s"/>
+      <x:c r="CR8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CS8"/>
+      <x:c r="CT8" s="10" t="s"/>
+      <x:c r="CU8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CV8"/>
+      <x:c r="CW8" s="10" t="s"/>
+      <x:c r="CX8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CY8" s="10" t="s"/>
+      <x:c r="CZ8"/>
+      <x:c r="DA8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DB8" s="10" t="s"/>
+      <x:c r="DC8"/>
+      <x:c r="DD8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DE8" s="10" t="s"/>
+      <x:c r="DF8"/>
+      <x:c r="DG8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DH8" s="10" t="s"/>
+      <x:c r="DI8"/>
+      <x:c r="DJ8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DK8" s="10" t="s"/>
+      <x:c r="DL8"/>
+      <x:c r="DM8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DN8" s="10" t="s"/>
+      <x:c r="DO8"/>
+      <x:c r="DP8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DQ8" s="10" t="s"/>
+      <x:c r="DR8"/>
+      <x:c r="DS8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DT8" s="10" t="s"/>
+      <x:c r="DU8"/>
+      <x:c r="DV8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DW8" s="10" t="s"/>
+      <x:c r="DX8"/>
+      <x:c r="DY8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DZ8" s="10" t="s"/>
+      <x:c r="EA8"/>
+      <x:c r="EB8">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC8" s="10" t="s"/>
+      <x:c r="ED8"/>
+      <x:c r="EE8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EF8" s="10" t="s"/>
+      <x:c r="EG8"/>
+      <x:c r="EH8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EI8" s="10" t="s"/>
+      <x:c r="EJ8"/>
+      <x:c r="EK8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EL8" s="10" t="s"/>
+      <x:c r="EM8"/>
+      <x:c r="EN8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EO8" s="10" t="s"/>
+      <x:c r="EP8"/>
+      <x:c r="EQ8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="ER8" s="10" t="s"/>
+      <x:c r="ES8"/>
+      <x:c r="ET8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EU8" s="10" t="s"/>
+      <x:c r="EV8"/>
+      <x:c r="EW8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EX8" s="10" t="s"/>
+      <x:c r="EY8"/>
+      <x:c r="EZ8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FA8" s="10" t="s"/>
+      <x:c r="FB8"/>
+      <x:c r="FC8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FD8" s="10" t="s"/>
+      <x:c r="FE8"/>
+      <x:c r="FF8">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FG8" s="10" t="s"/>
+      <x:c r="FH8"/>
+      <x:c r="FI8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FJ8" s="10" t="s"/>
+      <x:c r="FK8"/>
+      <x:c r="FL8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FM8" s="10" t="s"/>
+      <x:c r="FN8"/>
+      <x:c r="FO8">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FP8" s="10" t="s"/>
+      <x:c r="FQ8"/>
+      <x:c r="FR8">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS8" s="10" t="s"/>
+      <x:c r="FT8"/>
+      <x:c r="FU8">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FV8" s="10" t="s"/>
+      <x:c r="FW8"/>
+      <x:c r="FX8" s="10" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="FY8" s="10" t="s"/>
+      <x:c r="FZ8"/>
+      <x:c r="GA8" s="10" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="GB8" s="10" t="s"/>
+      <x:c r="GC8"/>
+      <x:c r="GD8" s="10" t="s"/>
+      <x:c r="GE8" s="10" t="s"/>
+      <x:c r="GF8"/>
+      <x:c r="GG8" s="10" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="GH8" s="10" t="s"/>
+      <x:c r="GI8"/>
+      <x:c r="GJ8" s="10" t="s"/>
+      <x:c r="GK8" s="10" t="s"/>
+      <x:c r="GL8"/>
+      <x:c r="GM8" s="10" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="GN8" s="10" t="s"/>
+      <x:c r="GO8"/>
+      <x:c r="GP8" s="10" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="GQ8" s="10" t="s"/>
+      <x:c r="GR8"/>
+      <x:c r="GS8" s="10" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="GT8" s="10" t="s"/>
+      <x:c r="GU8"/>
+    </x:row>
+    <x:row r="9" hidden="0">
+      <x:c r="A9">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="2">
+        <x:v>45959.6880324074</x:v>
+      </x:c>
+      <x:c r="C9" s="2">
+        <x:v>45959.7254050926</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="s"/>
+      <x:c r="F9"/>
+      <x:c r="G9" s="10" t="s"/>
+      <x:c r="H9" s="2"/>
+      <x:c r="I9" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J9"/>
+      <x:c r="K9" s="10" t="s"/>
+      <x:c r="L9" s="10" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="M9"/>
+      <x:c r="N9" s="10" t="s"/>
+      <x:c r="O9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P9"/>
+      <x:c r="Q9" s="10" t="s"/>
+      <x:c r="R9" s="10" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="S9"/>
+      <x:c r="T9" s="10" t="s"/>
+      <x:c r="U9"/>
+      <x:c r="V9" s="10" t="s"/>
+      <x:c r="W9" s="10" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="X9"/>
+      <x:c r="Y9" s="10" t="s"/>
+      <x:c r="Z9" s="10" t="s"/>
+      <x:c r="AA9"/>
+      <x:c r="AB9" s="10" t="s"/>
+      <x:c r="AC9"/>
+      <x:c r="AD9" s="10" t="s"/>
+      <x:c r="AE9" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AF9" s="10" t="s"/>
+      <x:c r="AG9"/>
+      <x:c r="AH9" s="10" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="AI9" s="10" t="s"/>
+      <x:c r="AJ9"/>
+      <x:c r="AK9" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AL9" s="10" t="s"/>
+      <x:c r="AM9"/>
+      <x:c r="AN9" s="10" t="s"/>
+      <x:c r="AO9" s="10" t="s"/>
+      <x:c r="AP9"/>
+      <x:c r="AQ9" s="10" t="s"/>
+      <x:c r="AR9" s="10" t="s"/>
+      <x:c r="AS9"/>
+      <x:c r="AT9" s="10" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="AU9" s="10" t="s"/>
+      <x:c r="AV9"/>
+      <x:c r="AW9" s="10" t="s"/>
+      <x:c r="AX9"/>
+      <x:c r="AY9" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="AZ9" s="10" t="s"/>
+      <x:c r="BA9"/>
+      <x:c r="BB9" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BC9"/>
+      <x:c r="BD9" s="10" t="s"/>
+      <x:c r="BE9" s="10" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="BF9"/>
+      <x:c r="BG9" s="10" t="s"/>
+      <x:c r="BH9"/>
+      <x:c r="BI9" s="10" t="s"/>
+      <x:c r="BJ9" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BK9"/>
+      <x:c r="BL9" s="10" t="s"/>
+      <x:c r="BM9" s="10" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="BN9"/>
+      <x:c r="BO9" s="10" t="s"/>
+      <x:c r="BP9"/>
+      <x:c r="BQ9" s="10" t="s"/>
+      <x:c r="BR9" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BS9"/>
+      <x:c r="BT9" s="10" t="s"/>
+      <x:c r="BU9" s="10" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="BV9"/>
+      <x:c r="BW9" s="10" t="s"/>
+      <x:c r="BX9"/>
+      <x:c r="BY9" s="10" t="s"/>
+      <x:c r="BZ9" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA9"/>
+      <x:c r="CB9" s="10" t="s"/>
+      <x:c r="CC9" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CD9"/>
+      <x:c r="CE9" s="10" t="s"/>
+      <x:c r="CF9" s="10" t="s"/>
+      <x:c r="CG9"/>
+      <x:c r="CH9" s="10" t="s"/>
+      <x:c r="CI9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CJ9"/>
+      <x:c r="CK9" s="10" t="s"/>
+      <x:c r="CL9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="CM9"/>
+      <x:c r="CN9" s="10" t="s"/>
+      <x:c r="CO9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CP9"/>
+      <x:c r="CQ9" s="10" t="s"/>
+      <x:c r="CR9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CS9"/>
+      <x:c r="CT9" s="10" t="s"/>
+      <x:c r="CU9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="CV9"/>
+      <x:c r="CW9" s="10" t="s"/>
+      <x:c r="CX9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CY9" s="10" t="s"/>
+      <x:c r="CZ9"/>
+      <x:c r="DA9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DB9" s="10" t="s"/>
+      <x:c r="DC9"/>
+      <x:c r="DD9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="DE9" s="10" t="s"/>
+      <x:c r="DF9"/>
+      <x:c r="DG9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="DH9" s="10" t="s"/>
+      <x:c r="DI9"/>
+      <x:c r="DJ9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DK9" s="10" t="s"/>
+      <x:c r="DL9"/>
+      <x:c r="DM9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DN9" s="10" t="s"/>
+      <x:c r="DO9"/>
+      <x:c r="DP9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="DQ9" s="10" t="s"/>
+      <x:c r="DR9"/>
+      <x:c r="DS9">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DT9" s="10" t="s"/>
+      <x:c r="DU9"/>
+      <x:c r="DV9">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DW9" s="10" t="s"/>
+      <x:c r="DX9"/>
+      <x:c r="DY9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="DZ9" s="10" t="s"/>
+      <x:c r="EA9"/>
+      <x:c r="EB9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EC9" s="10" t="s"/>
+      <x:c r="ED9"/>
+      <x:c r="EE9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="EF9" s="10" t="s"/>
+      <x:c r="EG9"/>
+      <x:c r="EH9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="EI9" s="10" t="s"/>
+      <x:c r="EJ9"/>
+      <x:c r="EK9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EL9" s="10" t="s"/>
+      <x:c r="EM9"/>
+      <x:c r="EN9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EO9" s="10" t="s"/>
+      <x:c r="EP9"/>
+      <x:c r="EQ9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="ER9" s="10" t="s"/>
+      <x:c r="ES9"/>
+      <x:c r="ET9">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="EU9" s="10" t="s"/>
+      <x:c r="EV9"/>
+      <x:c r="EW9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EX9" s="10" t="s"/>
+      <x:c r="EY9"/>
+      <x:c r="EZ9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FA9" s="10" t="s"/>
+      <x:c r="FB9"/>
+      <x:c r="FC9">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FD9" s="10" t="s"/>
+      <x:c r="FE9"/>
+      <x:c r="FF9">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="FG9" s="10" t="s"/>
+      <x:c r="FH9"/>
+      <x:c r="FI9">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FJ9" s="10" t="s"/>
+      <x:c r="FK9"/>
+      <x:c r="FL9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FM9" s="10" t="s"/>
+      <x:c r="FN9"/>
+      <x:c r="FO9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="FP9" s="10" t="s"/>
+      <x:c r="FQ9"/>
+      <x:c r="FR9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FS9" s="10" t="s"/>
+      <x:c r="FT9"/>
+      <x:c r="FU9">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FV9" s="10" t="s"/>
+      <x:c r="FW9"/>
+      <x:c r="FX9" s="10" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="FY9" s="10" t="s"/>
+      <x:c r="FZ9"/>
+      <x:c r="GA9" s="10" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="GB9" s="10" t="s"/>
+      <x:c r="GC9"/>
+      <x:c r="GD9" s="10" t="s"/>
+      <x:c r="GE9" s="10" t="s"/>
+      <x:c r="GF9"/>
+      <x:c r="GG9" s="10" t="s"/>
+      <x:c r="GH9" s="10" t="s"/>
+      <x:c r="GI9"/>
+      <x:c r="GJ9" s="10" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="GK9" s="10" t="s"/>
+      <x:c r="GL9"/>
+      <x:c r="GM9" s="10" t="s"/>
+      <x:c r="GN9" s="10" t="s"/>
+      <x:c r="GO9"/>
+      <x:c r="GP9" s="10" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="GQ9" s="10" t="s"/>
+      <x:c r="GR9"/>
+      <x:c r="GS9" s="10" t="s"/>
+      <x:c r="GT9" s="10" t="s"/>
+      <x:c r="GU9"/>
+    </x:row>
+    <x:row r="10" hidden="0">
+      <x:c r="A10">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="2">
+        <x:v>45959.7371296296</x:v>
+      </x:c>
+      <x:c r="C10" s="2">
+        <x:v>45959.7924537037</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="s">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="s"/>
+      <x:c r="F10"/>
+      <x:c r="G10" s="10" t="s"/>
+      <x:c r="H10" s="2"/>
+      <x:c r="I10" s="10" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="J10"/>
+      <x:c r="K10" s="10" t="s"/>
+      <x:c r="L10" s="10" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="M10"/>
+      <x:c r="N10" s="10" t="s"/>
+      <x:c r="O10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="P10"/>
+      <x:c r="Q10" s="10" t="s"/>
+      <x:c r="R10" s="10" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="S10"/>
+      <x:c r="T10" s="10" t="s"/>
+      <x:c r="U10"/>
+      <x:c r="V10" s="10" t="s"/>
+      <x:c r="W10" s="10" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="X10"/>
+      <x:c r="Y10" s="10" t="s"/>
+      <x:c r="Z10" s="10" t="s"/>
+      <x:c r="AA10"/>
+      <x:c r="AB10" s="10" t="s"/>
+      <x:c r="AC10"/>
+      <x:c r="AD10" s="10" t="s"/>
+      <x:c r="AE10" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AF10" s="10" t="s"/>
+      <x:c r="AG10"/>
+      <x:c r="AH10" s="10" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="AI10" s="10" t="s"/>
+      <x:c r="AJ10"/>
+      <x:c r="AK10" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="AL10" s="10" t="s"/>
+      <x:c r="AM10"/>
+      <x:c r="AN10" s="10" t="s"/>
+      <x:c r="AO10" s="10" t="s"/>
+      <x:c r="AP10"/>
+      <x:c r="AQ10" s="10" t="s"/>
+      <x:c r="AR10" s="10" t="s"/>
+      <x:c r="AS10"/>
+      <x:c r="AT10" s="10" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="AU10" s="10" t="s"/>
+      <x:c r="AV10"/>
+      <x:c r="AW10" s="10" t="s"/>
+      <x:c r="AX10"/>
+      <x:c r="AY10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="AZ10" s="10" t="s"/>
+      <x:c r="BA10"/>
+      <x:c r="BB10" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BC10"/>
+      <x:c r="BD10" s="10" t="s"/>
+      <x:c r="BE10" s="10" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="BF10"/>
+      <x:c r="BG10" s="10" t="s"/>
+      <x:c r="BH10"/>
+      <x:c r="BI10" s="10" t="s"/>
+      <x:c r="BJ10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BK10"/>
+      <x:c r="BL10" s="10" t="s"/>
+      <x:c r="BM10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BN10"/>
+      <x:c r="BO10" s="10" t="s"/>
+      <x:c r="BP10"/>
+      <x:c r="BQ10" s="10" t="s"/>
+      <x:c r="BR10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="BS10"/>
+      <x:c r="BT10" s="10" t="s"/>
+      <x:c r="BU10" s="10" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="BV10"/>
+      <x:c r="BW10" s="10" t="s"/>
+      <x:c r="BX10"/>
+      <x:c r="BY10" s="10" t="s"/>
+      <x:c r="BZ10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CA10"/>
+      <x:c r="CB10" s="10" t="s"/>
+      <x:c r="CC10" s="10" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="CD10"/>
+      <x:c r="CE10" s="10" t="s"/>
+      <x:c r="CF10" s="10" t="s"/>
+      <x:c r="CG10"/>
+      <x:c r="CH10" s="10" t="s"/>
+      <x:c r="CI10">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CJ10"/>
+      <x:c r="CK10" s="10" t="s"/>
+      <x:c r="CL10">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CM10"/>
+      <x:c r="CN10" s="10" t="s"/>
+      <x:c r="CO10">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="CP10"/>
+      <x:c r="CQ10" s="10" t="s"/>
+      <x:c r="CR10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="CS10"/>
+      <x:c r="CT10" s="10" t="s"/>
+      <x:c r="CU10">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="CV10"/>
+      <x:c r="CW10" s="10" t="s"/>
+      <x:c r="CX10">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="CY10" s="10" t="s"/>
+      <x:c r="CZ10"/>
+      <x:c r="DA10">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DB10" s="10" t="s"/>
+      <x:c r="DC10"/>
+      <x:c r="DD10">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DE10" s="10" t="s"/>
+      <x:c r="DF10"/>
+      <x:c r="DG10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DH10" s="10" t="s"/>
+      <x:c r="DI10"/>
+      <x:c r="DJ10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="DK10" s="10" t="s"/>
+      <x:c r="DL10"/>
+      <x:c r="DM10">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DN10" s="10" t="s"/>
+      <x:c r="DO10"/>
+      <x:c r="DP10">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="DQ10" s="10" t="s"/>
+      <x:c r="DR10"/>
+      <x:c r="DS10">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DT10" s="10" t="s"/>
+      <x:c r="DU10"/>
+      <x:c r="DV10">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="DW10" s="10" t="s"/>
+      <x:c r="DX10"/>
+      <x:c r="DY10">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="DZ10" s="10" t="s"/>
+      <x:c r="EA10"/>
+      <x:c r="EB10">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="EC10" s="10" t="s"/>
+      <x:c r="ED10"/>
+      <x:c r="EE10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EF10" s="10" t="s"/>
+      <x:c r="EG10"/>
+      <x:c r="EH10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="EI10" s="10" t="s"/>
+      <x:c r="EJ10"/>
+      <x:c r="EK10">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EL10" s="10" t="s"/>
+      <x:c r="EM10"/>
+      <x:c r="EN10">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="EO10" s="10" t="s"/>
+      <x:c r="EP10"/>
+      <x:c r="EQ10">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="ER10" s="10" t="s"/>
+      <x:c r="ES10"/>
+      <x:c r="ET10">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="EU10" s="10" t="s"/>
+      <x:c r="EV10"/>
+      <x:c r="EW10">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="EX10" s="10" t="s"/>
+      <x:c r="EY10"/>
+      <x:c r="EZ10">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="FA10" s="10" t="s"/>
+      <x:c r="FB10"/>
+      <x:c r="FC10">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="FD10" s="10" t="s"/>
+      <x:c r="FE10"/>
+      <x:c r="FF10">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="FG10" s="10" t="s"/>
+      <x:c r="FH10"/>
+      <x:c r="FI10">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FJ10" s="10" t="s"/>
+      <x:c r="FK10"/>
+      <x:c r="FL10">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FM10" s="10" t="s"/>
+      <x:c r="FN10"/>
+      <x:c r="FO10">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="FP10" s="10" t="s"/>
+      <x:c r="FQ10"/>
+      <x:c r="FR10">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FS10" s="10" t="s"/>
+      <x:c r="FT10"/>
+      <x:c r="FU10">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="FV10" s="10" t="s"/>
+      <x:c r="FW10"/>
+      <x:c r="FX10" s="10" t="s"/>
+      <x:c r="FY10" s="10" t="s"/>
+      <x:c r="FZ10"/>
+      <x:c r="GA10" s="10" t="s"/>
+      <x:c r="GB10" s="10" t="s"/>
+      <x:c r="GC10"/>
+      <x:c r="GD10" s="10" t="s"/>
+      <x:c r="GE10" s="10" t="s"/>
+      <x:c r="GF10"/>
+      <x:c r="GG10" s="10" t="s"/>
+      <x:c r="GH10" s="10" t="s"/>
+      <x:c r="GI10"/>
+      <x:c r="GJ10" s="10" t="s"/>
+      <x:c r="GK10" s="10" t="s"/>
+      <x:c r="GL10"/>
+      <x:c r="GM10" s="10" t="s"/>
+      <x:c r="GN10" s="10" t="s"/>
+      <x:c r="GO10"/>
+      <x:c r="GP10" s="10" t="s"/>
+      <x:c r="GQ10" s="10" t="s"/>
+      <x:c r="GR10"/>
+      <x:c r="GS10" s="10" t="s"/>
+      <x:c r="GT10" s="10" t="s"/>
+      <x:c r="GU10"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="Rc3162834260c4d69"/>
+    <x:tablePart r:id="Rc12a975297544112"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>